<commit_message>
Confirm the textbook citation: Larson and Hostetler, Thomson Brooks/Cole, 2009
Record the coauthor, publisher, year, ISBN-13 and ISBN-10, and the
Pre-AP National Student Edition variant as confirmed by the owner, flip
the verified flags, and include the edition note and ISBN in the
generated citation. Regenerate the index, tracker, and checklist.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LvqXmfNy6dNh6SXPzmJwF
</commit_message>
<xml_diff>
--- a/dist/progress-tracker.xlsx
+++ b/dist/progress-tracker.xlsx
@@ -17623,7 +17623,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ron Larson. *Precalculus with Limits*, 2nd ed. Brooks/Cole, Cengage Learning, 2011.</t>
+          <t>Ron Larson and Robert P. Hostetler. *Precalculus with Limits*, 2nd ed. (Pre-AP National Student Edition) Thomson Brooks/Cole, 2009. ISBN 978-0-538-73659-6.</t>
         </is>
       </c>
     </row>
@@ -17647,7 +17647,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>git 6614701</t>
+          <t>git b6c7ce7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Address CodeRabbit review: plain-text citation, loader and validator guards
Return the citation as plain text and add Markdown emphasis only in the
index, so the About sheet and PDF footer no longer show asterisks. Let a
unit with no name reach the validator instead of raising KeyError.
Require a coverage note on every mapped unit. Store any catalog text
beginning with "=" as text, never as a formula. Fix stale design text:
the By section sheet name, chapter summaries as a top-level list,
mapping scope chapters 1 through 3, and a verifier field in the study
guide answer-verification record. Tests added for each code change.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LvqXmfNy6dNh6SXPzmJwF
</commit_message>
<xml_diff>
--- a/dist/progress-tracker.xlsx
+++ b/dist/progress-tracker.xlsx
@@ -17623,7 +17623,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ron Larson and Robert P. Hostetler. *Precalculus with Limits*, 2nd ed. (Pre-AP National Student Edition) Thomson Brooks/Cole, 2009. ISBN 978-0-538-73659-6.</t>
+          <t>Ron Larson and Robert P. Hostetler. Precalculus with Limits, 2nd ed. (Pre-AP National Student Edition) Thomson Brooks/Cole, 2009. ISBN 978-0-538-73659-6.</t>
         </is>
       </c>
     </row>
@@ -17647,7 +17647,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>git b6c7ce7</t>
+          <t>git 3b8bf92</t>
         </is>
       </c>
     </row>

</xml_diff>